<commit_message>
&& - 83454101 (2 часть) от 20.11.2025 https://meshok.net/
</commit_message>
<xml_diff>
--- a/Collections/EURO/Monaco/#EURO#Monaco#Commemorative#[2007-present]#UNC.xlsx
+++ b/Collections/EURO/Monaco/#EURO#Monaco#Commemorative#[2007-present]#UNC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lord_Alexator\Documents\CoinCollection\Collections\EURO\Monaco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166F2E2F-80F5-4A91-A17B-D4ECBB6981CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF5F521-D37D-464F-87F2-3D0545B2764A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="55">
   <si>
     <t>Year</t>
   </si>
@@ -245,6 +245,9 @@
   </si>
   <si>
     <t>County of Carladès</t>
+  </si>
+  <si>
+    <t>Marquisate of Baux</t>
   </si>
 </sst>
 </file>
@@ -560,7 +563,7 @@
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -585,6 +588,14 @@
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9BE5FF"/>
+          <bgColor rgb="FF9BE5FF"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -942,7 +953,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.6328125" style="12" customWidth="1"/>
@@ -1505,8 +1516,8 @@
       <c r="G20" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="H20" s="24" t="s">
-        <v>4</v>
+      <c r="H20" s="28">
+        <v>1</v>
       </c>
       <c r="I20" s="11" t="str">
         <f t="shared" si="6"/>
@@ -1566,6 +1577,34 @@
       </c>
       <c r="I22" s="11" t="str">
         <f t="shared" ref="I22" si="7">IF(OR(AND(H22&gt;1,H22&lt;&gt;"-")),"Can exchange","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="22">
+        <v>2025</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G23" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="H23" s="28">
+        <v>1</v>
+      </c>
+      <c r="I23" s="11" t="str">
+        <f t="shared" ref="I23" si="8">IF(OR(AND(H23&gt;1,H23&lt;&gt;"-")),"Can exchange","")</f>
         <v/>
       </c>
     </row>
@@ -1577,12 +1616,12 @@
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="H7:H9">
-    <cfRule type="containsText" dxfId="12" priority="29" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="13" priority="33" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H7))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:H9">
-    <cfRule type="colorScale" priority="30">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -1594,11 +1633,45 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
-    <cfRule type="containsText" dxfId="11" priority="17" operator="containsText" text="*-">
+    <cfRule type="containsText" dxfId="12" priority="21" operator="containsText" text="*-">
       <formula>NOT(ISERROR(SEARCH(("*-"),(H11))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="containsText" dxfId="11" priority="19" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12:H16 H18 H22">
+    <cfRule type="containsText" dxfId="10" priority="17" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H12))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12:H16 H18 H22">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -1610,13 +1683,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3">
-    <cfRule type="containsText" dxfId="10" priority="15" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H3))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3">
-    <cfRule type="colorScale" priority="16">
+  <conditionalFormatting sqref="H4:H6">
+    <cfRule type="containsText" dxfId="9" priority="23" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H4:H6">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -1627,12 +1700,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:H16 H18 H20 H22">
-    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H12))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H12:H16 H18 H20 H22">
+  <conditionalFormatting sqref="H17">
+    <cfRule type="containsText" dxfId="8" priority="13" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -1644,13 +1717,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4:H6">
-    <cfRule type="containsText" dxfId="8" priority="19" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H4))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H4:H6">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="H10">
+    <cfRule type="containsText" dxfId="7" priority="11" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H10))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H10">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="formula" val="0"/>
         <cfvo type="formula" val="1"/>
@@ -1661,29 +1734,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H17">
-    <cfRule type="containsText" dxfId="7" priority="9" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H17))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H17">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="formula" val="0"/>
-        <cfvo type="formula" val="1"/>
-        <cfvo type="formula" val="10"/>
-        <color rgb="FFFF9F9F"/>
-        <color rgb="FFD1E0B2"/>
-        <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
+  <conditionalFormatting sqref="H21">
     <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H10))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H21))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H21">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -1695,12 +1751,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
+  <conditionalFormatting sqref="H19">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="*-">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H19))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="formula" val="1"/>
+        <cfvo type="formula" val="10"/>
+        <color rgb="FFFF9F9F"/>
+        <color rgb="FFD1E0B2"/>
+        <color rgb="FF00B050"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
     <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H21))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H20))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="formula" val="0"/>
@@ -1712,12 +1785,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H19">
+  <conditionalFormatting sqref="H23">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="*-">
-      <formula>NOT(ISERROR(SEARCH(("*-"),(H19))))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H19">
+      <formula>NOT(ISERROR(SEARCH(("*-"),(H23))))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="formula" val="0"/>

</xml_diff>